<commit_message>
Remove birthday-celebration mentions and the Source column
Replaced all 19 "birthday" (عيد ميلاد) mentions across the 300 and 700
sentence sets with "graduation" (تخرج) as a neutral occasion -- only the
Arabic occasion wording changed, English terms/word counts are untouched.
Swept both files for other potentially objectionable content (alcohol,
gambling, dating, pork); none found.

Also dropped the Source column from the combined 1000 workbook per request.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155UPXv8Dk7askKg634TkFB
</commit_message>
<xml_diff>
--- a/arabic_english_codeswitching_700_new.xlsx
+++ b/arabic_english_codeswitching_700_new.xlsx
@@ -536,7 +536,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بعيد ميلادها في مطعم وسط Colours، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Colours، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت donut وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت donut وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1233,7 +1233,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت chocolate lava cake وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت chocolate lava cake وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بعيد ميلادها في مطعم وسط Avenues، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Avenues، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -3477,7 +3477,7 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت tiramisu وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت tiramisu وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
@@ -3494,7 +3494,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>أهدوني شنطة Chanel في عيد ميلادي وكانت هدية فخمة، ما توقعت حد يهديني شي بهالمستوى.</t>
+          <t>أهدوني شنطة Chanel في تخرجي وكانت هدية فخمة، ما توقعت حد يهديني شي بهالمستوى.</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -5109,7 +5109,7 @@
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>أهدوني شنطة Gucci في عيد ميلادي وكانت هدية فخمة، ما توقعت حد يهديني شي بهالمستوى.</t>
+          <t>أهدوني شنطة Gucci في تخرجي وكانت هدية فخمة، ما توقعت حد يهديني شي بهالمستوى.</t>
         </is>
       </c>
       <c r="B276" s="3" t="inlineStr">
@@ -6078,7 +6078,7 @@
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت ice cream sundae وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت ice cream sundae وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B333" s="3" t="inlineStr">
@@ -6282,7 +6282,7 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت brownie وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت brownie وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B345" s="3" t="inlineStr">
@@ -6435,7 +6435,7 @@
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بعيد ميلادها في مطعم وسط Uptown، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Uptown، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B354" s="3" t="inlineStr">
@@ -6724,7 +6724,7 @@
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بعيد ميلادها في مطعم وسط Boulevard World، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Boulevard World، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B371" s="3" t="inlineStr">
@@ -7523,7 +7523,7 @@
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بعيد ميلادها في مطعم وسط Downtown، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Downtown، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B418" s="3" t="inlineStr">
@@ -7846,7 +7846,7 @@
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت bubble tea وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت bubble tea وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B437" s="3" t="inlineStr">
@@ -9291,7 +9291,7 @@
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت chai latte وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت chai latte وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B522" s="3" t="inlineStr">
@@ -9325,7 +9325,7 @@
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>أهدوني ساعة Rolex في عيد ميلادي وكانت هدية فخمة، ولين الحين أحافظ عليها مثل الذهب.</t>
+          <t>أهدوني ساعة Rolex في تخرجي وكانت هدية فخمة، ولين الحين أحافظ عليها مثل الذهب.</t>
         </is>
       </c>
       <c r="B524" s="3" t="inlineStr">
@@ -9376,7 +9376,7 @@
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>أهدوني شنطة Louis Vuitton في عيد ميلادي وكانت هدية فخمة، ما توقعت حد يهديني شي بهالمستوى.</t>
+          <t>أهدوني شنطة Louis Vuitton في تخرجي وكانت هدية فخمة، ما توقعت حد يهديني شي بهالمستوى.</t>
         </is>
       </c>
       <c r="B527" s="3" t="inlineStr">
@@ -10226,7 +10226,7 @@
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بعيد ميلادها في مطعم وسط KAFD، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط KAFD، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B577" s="3" t="inlineStr">
@@ -11824,7 +11824,7 @@
     <row r="671">
       <c r="A671" s="2" t="inlineStr">
         <is>
-          <t>في عيد ميلادي طلبت hotdog وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
+          <t>في تخرجي طلبت hotdog وكيكة من نفس المطعم لأنهم أفضل مكان جربته بصراحة.</t>
         </is>
       </c>
       <c r="B671" s="3" t="inlineStr">

</xml_diff>